<commit_message>
Add Parcours autonome in template
</commit_message>
<xml_diff>
--- a/TimesheetFs/Timesheet-Template.xlsx
+++ b/TimesheetFs/Timesheet-Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Perso\Taggl\TimesheetFs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD81471C-5B5D-4D7D-A031-B85849F0009F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{569E2994-7B5C-4353-B834-C2D1EB1F7906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="4" xr2:uid="{FB794F17-9F1B-438B-B219-D10D95E788D4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{FB794F17-9F1B-438B-B219-D10D95E788D4}"/>
   </bookViews>
   <sheets>
     <sheet name="Configuration" sheetId="5" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="156">
   <si>
     <r>
       <t>1. Onglet "</t>
@@ -786,6 +786,12 @@
   </si>
   <si>
     <t>Wavenet</t>
+  </si>
+  <si>
+    <t>PARCE-PAUTO</t>
+  </si>
+  <si>
+    <t>Parcours autonome</t>
   </si>
 </sst>
 </file>
@@ -2676,19 +2682,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{534EC4EE-AC4C-4AAA-B056-D5CBC744E76C}">
   <dimension ref="A1:AL64"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="34" customWidth="1"/>
-    <col min="2" max="2" width="3.453125" customWidth="1"/>
-    <col min="3" max="3" width="29.54296875" customWidth="1"/>
-    <col min="4" max="4" width="65.81640625" customWidth="1"/>
-    <col min="5" max="5" width="3.453125" style="34" customWidth="1"/>
+    <col min="2" max="2" width="3.42578125" customWidth="1"/>
+    <col min="3" max="3" width="29.5703125" customWidth="1"/>
+    <col min="4" max="4" width="65.85546875" customWidth="1"/>
+    <col min="5" max="5" width="3.42578125" style="34" customWidth="1"/>
     <col min="6" max="38" width="0" hidden="1" customWidth="1"/>
-    <col min="39" max="16384" width="9.1796875" hidden="1"/>
+    <col min="39" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="34" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:34" s="34" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B2" s="120" t="s">
         <v>0</v>
       </c>
@@ -2723,7 +2729,7 @@
       <c r="AG2" s="61"/>
       <c r="AH2" s="61"/>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B3" s="99"/>
       <c r="C3" s="126" t="s">
         <v>1</v>
@@ -2758,7 +2764,7 @@
       <c r="AG3" s="61"/>
       <c r="AH3" s="61"/>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B4" s="99"/>
       <c r="C4" s="126" t="s">
         <v>2</v>
@@ -2793,7 +2799,7 @@
       <c r="AG4" s="61"/>
       <c r="AH4" s="61"/>
     </row>
-    <row r="5" spans="1:34" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:34" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="62"/>
       <c r="C5" s="123" t="s">
         <v>3</v>
@@ -2828,7 +2834,7 @@
       <c r="AG5" s="61"/>
       <c r="AH5" s="61"/>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B6" s="125" t="s">
         <v>4</v>
       </c>
@@ -2863,7 +2869,7 @@
       <c r="AG6" s="61"/>
       <c r="AH6" s="61"/>
     </row>
-    <row r="7" spans="1:34" s="97" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:34" s="97" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="95"/>
       <c r="B7" s="96"/>
       <c r="C7" s="123" t="s">
@@ -2872,7 +2878,7 @@
       <c r="D7" s="124"/>
       <c r="E7" s="95"/>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B8" s="99"/>
       <c r="C8" s="126" t="s">
         <v>6</v>
@@ -2907,7 +2913,7 @@
       <c r="AG8" s="61"/>
       <c r="AH8" s="61"/>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B9" s="62"/>
       <c r="C9" s="123" t="s">
         <v>7</v>
@@ -2942,7 +2948,7 @@
       <c r="AG9" s="61"/>
       <c r="AH9" s="61"/>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="B10" s="125" t="s">
         <v>8</v>
       </c>
@@ -2977,7 +2983,7 @@
       <c r="AG10" s="61"/>
       <c r="AH10" s="61"/>
     </row>
-    <row r="11" spans="1:34" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:34" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="63"/>
       <c r="C11" s="136" t="s">
         <v>9</v>
@@ -3012,8 +3018,8 @@
       <c r="AG11" s="61"/>
       <c r="AH11" s="61"/>
     </row>
-    <row r="12" spans="1:34" s="34" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="13" spans="1:34" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:34" s="34" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:34" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="128" t="s">
         <v>10</v>
       </c>
@@ -3022,21 +3028,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:34" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B14" s="130" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="131"/>
       <c r="D14" s="102"/>
     </row>
-    <row r="15" spans="1:34" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:34" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="132" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="133"/>
       <c r="D15" s="65"/>
     </row>
-    <row r="16" spans="1:34" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:34" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B16" s="132" t="s">
         <v>13</v>
       </c>
@@ -3045,7 +3051,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="134" t="s">
         <v>14</v>
       </c>
@@ -3054,7 +3060,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="19" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="128" t="s">
         <v>15</v>
       </c>
@@ -3063,7 +3069,7 @@
         <v>1.6666666666666667</v>
       </c>
     </row>
-    <row r="19" spans="2:4" s="34" customFormat="1" ht="19" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:4" s="34" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="128" t="s">
         <v>16</v>
       </c>
@@ -3073,59 +3079,59 @@
         <v>0.33333333333333337</v>
       </c>
     </row>
-    <row r="20" spans="2:4" s="34" customFormat="1" x14ac:dyDescent="0.35"/>
-    <row r="21" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="22" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="23" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="24" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="25" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="27" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="28" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="29" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="31" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="32" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="33" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="34" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" s="34" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="2:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="34" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="34" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D35" s="34" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="37" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="38" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="40" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="41" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="42" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="43" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="44" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="45" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="46" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="47" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="48" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="49" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="50" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="51" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="52" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="53" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="54" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="55" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="56" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="57" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="58" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="59" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="60" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="61" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="62" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="63" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="64" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="36" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="4:4" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="49" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="50" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="51" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="52" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="53" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="54" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="55" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="56" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="57" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="58" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="59" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="60" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="61" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="62" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="63" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="64" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="B18:C18"/>
@@ -3169,18 +3175,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A0187C1-7D96-4BCF-AD52-481055EFB1E2}">
   <dimension ref="A1:AL140"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.7265625" style="34" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.26953125" customWidth="1"/>
-    <col min="4" max="34" width="6.1796875" style="59" customWidth="1"/>
-    <col min="35" max="35" width="3.26953125" style="34" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="34" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.28515625" customWidth="1"/>
+    <col min="4" max="34" width="6.140625" style="59" customWidth="1"/>
+    <col min="35" max="35" width="3.28515625" style="34" customWidth="1"/>
     <col min="36" max="38" width="0" style="34" hidden="1" customWidth="1"/>
-    <col min="39" max="16384" width="9.1796875" hidden="1"/>
+    <col min="39" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:35" s="34" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:35" s="34" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D1" s="60"/>
       <c r="E1" s="60"/>
       <c r="F1" s="60"/>
@@ -3213,7 +3219,7 @@
       <c r="AG1" s="60"/>
       <c r="AH1" s="60"/>
     </row>
-    <row r="2" spans="2:35" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:35" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>19</v>
       </c>
@@ -3346,7 +3352,7 @@
       </c>
       <c r="AI2" s="2"/>
     </row>
-    <row r="3" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B3" s="38"/>
       <c r="C3" s="47" t="s">
         <v>21</v>
@@ -3384,7 +3390,7 @@
       <c r="AH3" s="52"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B4" s="39"/>
       <c r="C4" s="48" t="s">
         <v>22</v>
@@ -3422,7 +3428,7 @@
       <c r="AH4" s="55"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B5" s="39"/>
       <c r="C5" s="48" t="s">
         <v>23</v>
@@ -3460,7 +3466,7 @@
       <c r="AH5" s="55"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" spans="2:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:35" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="40"/>
       <c r="C6" s="49" t="s">
         <v>24</v>
@@ -3498,7 +3504,7 @@
       <c r="AH6" s="58"/>
       <c r="AI6" s="2"/>
     </row>
-    <row r="7" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B7" s="41"/>
       <c r="C7" s="42" t="str">
         <f>IF(ISBLANK(B7),"",VLOOKUP(B7,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3536,7 +3542,7 @@
       <c r="AG7" s="51"/>
       <c r="AH7" s="52"/>
     </row>
-    <row r="8" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B8" s="43"/>
       <c r="C8" s="44" t="str">
         <f>IF(ISBLANK(B8),"",VLOOKUP(B8,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3574,7 +3580,7 @@
       <c r="AG8" s="54"/>
       <c r="AH8" s="55"/>
     </row>
-    <row r="9" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B9" s="43"/>
       <c r="C9" s="44" t="str">
         <f>IF(ISBLANK(B9),"",VLOOKUP(B9,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3612,7 +3618,7 @@
       <c r="AG9" s="54"/>
       <c r="AH9" s="55"/>
     </row>
-    <row r="10" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B10" s="43"/>
       <c r="C10" s="44" t="str">
         <f>IF(ISBLANK(B10),"",VLOOKUP(B10,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3650,7 +3656,7 @@
       <c r="AG10" s="54"/>
       <c r="AH10" s="55"/>
     </row>
-    <row r="11" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B11" s="43"/>
       <c r="C11" s="44" t="str">
         <f>IF(ISBLANK(B11),"",VLOOKUP(B11,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3688,7 +3694,7 @@
       <c r="AG11" s="54"/>
       <c r="AH11" s="55"/>
     </row>
-    <row r="12" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B12" s="43"/>
       <c r="C12" s="44" t="str">
         <f>IF(ISBLANK(B12),"",VLOOKUP(B12,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3726,7 +3732,7 @@
       <c r="AG12" s="54"/>
       <c r="AH12" s="55"/>
     </row>
-    <row r="13" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B13" s="43"/>
       <c r="C13" s="44" t="str">
         <f>IF(ISBLANK(B13),"",VLOOKUP(B13,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3764,7 +3770,7 @@
       <c r="AG13" s="54"/>
       <c r="AH13" s="55"/>
     </row>
-    <row r="14" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B14" s="43"/>
       <c r="C14" s="44" t="str">
         <f>IF(ISBLANK(B14),"",VLOOKUP(B14,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3802,7 +3808,7 @@
       <c r="AG14" s="54"/>
       <c r="AH14" s="55"/>
     </row>
-    <row r="15" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B15" s="43"/>
       <c r="C15" s="44" t="str">
         <f>IF(ISBLANK(B15),"",VLOOKUP(B15,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3840,7 +3846,7 @@
       <c r="AG15" s="54"/>
       <c r="AH15" s="55"/>
     </row>
-    <row r="16" spans="2:35" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B16" s="43"/>
       <c r="C16" s="44" t="str">
         <f>IF(ISBLANK(B16),"",VLOOKUP(B16,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3878,7 +3884,7 @@
       <c r="AG16" s="54"/>
       <c r="AH16" s="55"/>
     </row>
-    <row r="17" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B17" s="43"/>
       <c r="C17" s="44" t="str">
         <f>IF(ISBLANK(B17),"",VLOOKUP(B17,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3916,7 +3922,7 @@
       <c r="AG17" s="54"/>
       <c r="AH17" s="55"/>
     </row>
-    <row r="18" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B18" s="43"/>
       <c r="C18" s="44" t="str">
         <f>IF(ISBLANK(B18),"",VLOOKUP(B18,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3954,7 +3960,7 @@
       <c r="AG18" s="54"/>
       <c r="AH18" s="55"/>
     </row>
-    <row r="19" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B19" s="43"/>
       <c r="C19" s="44" t="str">
         <f>IF(ISBLANK(B19),"",VLOOKUP(B19,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -3992,7 +3998,7 @@
       <c r="AG19" s="54"/>
       <c r="AH19" s="55"/>
     </row>
-    <row r="20" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B20" s="43"/>
       <c r="C20" s="44" t="str">
         <f>IF(ISBLANK(B20),"",VLOOKUP(B20,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4030,7 +4036,7 @@
       <c r="AG20" s="54"/>
       <c r="AH20" s="55"/>
     </row>
-    <row r="21" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B21" s="43"/>
       <c r="C21" s="44" t="str">
         <f>IF(ISBLANK(B21),"",VLOOKUP(B21,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4068,7 +4074,7 @@
       <c r="AG21" s="54"/>
       <c r="AH21" s="55"/>
     </row>
-    <row r="22" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B22" s="43"/>
       <c r="C22" s="44" t="str">
         <f>IF(ISBLANK(B22),"",VLOOKUP(B22,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4106,7 +4112,7 @@
       <c r="AG22" s="54"/>
       <c r="AH22" s="55"/>
     </row>
-    <row r="23" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B23" s="43"/>
       <c r="C23" s="44" t="str">
         <f>IF(ISBLANK(B23),"",VLOOKUP(B23,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4144,7 +4150,7 @@
       <c r="AG23" s="54"/>
       <c r="AH23" s="55"/>
     </row>
-    <row r="24" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B24" s="43"/>
       <c r="C24" s="44" t="str">
         <f>IF(ISBLANK(B24),"",VLOOKUP(B24,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4182,7 +4188,7 @@
       <c r="AG24" s="54"/>
       <c r="AH24" s="55"/>
     </row>
-    <row r="25" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B25" s="43"/>
       <c r="C25" s="44" t="str">
         <f>IF(ISBLANK(B25),"",VLOOKUP(B25,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4220,7 +4226,7 @@
       <c r="AG25" s="54"/>
       <c r="AH25" s="55"/>
     </row>
-    <row r="26" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B26" s="43"/>
       <c r="C26" s="44" t="str">
         <f>IF(ISBLANK(B26),"",VLOOKUP(B26,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4258,7 +4264,7 @@
       <c r="AG26" s="54"/>
       <c r="AH26" s="55"/>
     </row>
-    <row r="27" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B27" s="43"/>
       <c r="C27" s="44" t="str">
         <f>IF(ISBLANK(B27),"",VLOOKUP(B27,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4296,7 +4302,7 @@
       <c r="AG27" s="54"/>
       <c r="AH27" s="55"/>
     </row>
-    <row r="28" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B28" s="43"/>
       <c r="C28" s="44" t="str">
         <f>IF(ISBLANK(B28),"",VLOOKUP(B28,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4334,7 +4340,7 @@
       <c r="AG28" s="54"/>
       <c r="AH28" s="55"/>
     </row>
-    <row r="29" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B29" s="43"/>
       <c r="C29" s="44" t="str">
         <f>IF(ISBLANK(B29),"",VLOOKUP(B29,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4372,7 +4378,7 @@
       <c r="AG29" s="54"/>
       <c r="AH29" s="55"/>
     </row>
-    <row r="30" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B30" s="43"/>
       <c r="C30" s="44" t="str">
         <f>IF(ISBLANK(B30),"",VLOOKUP(B30,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4410,7 +4416,7 @@
       <c r="AG30" s="54"/>
       <c r="AH30" s="55"/>
     </row>
-    <row r="31" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B31" s="43"/>
       <c r="C31" s="44" t="str">
         <f>IF(ISBLANK(B31),"",VLOOKUP(B31,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4448,7 +4454,7 @@
       <c r="AG31" s="54"/>
       <c r="AH31" s="55"/>
     </row>
-    <row r="32" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B32" s="43"/>
       <c r="C32" s="44" t="str">
         <f>IF(ISBLANK(B32),"",VLOOKUP(B32,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4486,7 +4492,7 @@
       <c r="AG32" s="54"/>
       <c r="AH32" s="55"/>
     </row>
-    <row r="33" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B33" s="43"/>
       <c r="C33" s="44" t="str">
         <f>IF(ISBLANK(B33),"",VLOOKUP(B33,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4524,7 +4530,7 @@
       <c r="AG33" s="54"/>
       <c r="AH33" s="55"/>
     </row>
-    <row r="34" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B34" s="43"/>
       <c r="C34" s="44" t="str">
         <f>IF(ISBLANK(B34),"",VLOOKUP(B34,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4562,7 +4568,7 @@
       <c r="AG34" s="54"/>
       <c r="AH34" s="55"/>
     </row>
-    <row r="35" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B35" s="43"/>
       <c r="C35" s="44" t="str">
         <f>IF(ISBLANK(B35),"",VLOOKUP(B35,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4600,7 +4606,7 @@
       <c r="AG35" s="54"/>
       <c r="AH35" s="55"/>
     </row>
-    <row r="36" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B36" s="43"/>
       <c r="C36" s="44" t="str">
         <f>IF(ISBLANK(B36),"",VLOOKUP(B36,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4638,7 +4644,7 @@
       <c r="AG36" s="54"/>
       <c r="AH36" s="55"/>
     </row>
-    <row r="37" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B37" s="43"/>
       <c r="C37" s="44" t="str">
         <f>IF(ISBLANK(B37),"",VLOOKUP(B37,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4676,7 +4682,7 @@
       <c r="AG37" s="54"/>
       <c r="AH37" s="55"/>
     </row>
-    <row r="38" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B38" s="43"/>
       <c r="C38" s="44" t="str">
         <f>IF(ISBLANK(B38),"",VLOOKUP(B38,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4714,7 +4720,7 @@
       <c r="AG38" s="54"/>
       <c r="AH38" s="55"/>
     </row>
-    <row r="39" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B39" s="43"/>
       <c r="C39" s="44" t="str">
         <f>IF(ISBLANK(B39),"",VLOOKUP(B39,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4752,7 +4758,7 @@
       <c r="AG39" s="54"/>
       <c r="AH39" s="55"/>
     </row>
-    <row r="40" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B40" s="43"/>
       <c r="C40" s="44" t="str">
         <f>IF(ISBLANK(B40),"",VLOOKUP(B40,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4790,7 +4796,7 @@
       <c r="AG40" s="54"/>
       <c r="AH40" s="55"/>
     </row>
-    <row r="41" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B41" s="43"/>
       <c r="C41" s="44" t="str">
         <f>IF(ISBLANK(B41),"",VLOOKUP(B41,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4828,7 +4834,7 @@
       <c r="AG41" s="54"/>
       <c r="AH41" s="55"/>
     </row>
-    <row r="42" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B42" s="43"/>
       <c r="C42" s="44" t="str">
         <f>IF(ISBLANK(B42),"",VLOOKUP(B42,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4866,7 +4872,7 @@
       <c r="AG42" s="54"/>
       <c r="AH42" s="55"/>
     </row>
-    <row r="43" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B43" s="43"/>
       <c r="C43" s="44" t="str">
         <f>IF(ISBLANK(B43),"",VLOOKUP(B43,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4904,7 +4910,7 @@
       <c r="AG43" s="54"/>
       <c r="AH43" s="55"/>
     </row>
-    <row r="44" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B44" s="43"/>
       <c r="C44" s="44" t="str">
         <f>IF(ISBLANK(B44),"",VLOOKUP(B44,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4942,7 +4948,7 @@
       <c r="AG44" s="54"/>
       <c r="AH44" s="55"/>
     </row>
-    <row r="45" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B45" s="43"/>
       <c r="C45" s="44" t="str">
         <f>IF(ISBLANK(B45),"",VLOOKUP(B45,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -4980,7 +4986,7 @@
       <c r="AG45" s="54"/>
       <c r="AH45" s="55"/>
     </row>
-    <row r="46" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B46" s="43"/>
       <c r="C46" s="44" t="str">
         <f>IF(ISBLANK(B46),"",VLOOKUP(B46,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5018,7 +5024,7 @@
       <c r="AG46" s="54"/>
       <c r="AH46" s="55"/>
     </row>
-    <row r="47" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B47" s="43"/>
       <c r="C47" s="44" t="str">
         <f>IF(ISBLANK(B47),"",VLOOKUP(B47,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5056,7 +5062,7 @@
       <c r="AG47" s="54"/>
       <c r="AH47" s="55"/>
     </row>
-    <row r="48" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B48" s="43"/>
       <c r="C48" s="44" t="str">
         <f>IF(ISBLANK(B48),"",VLOOKUP(B48,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5094,7 +5100,7 @@
       <c r="AG48" s="54"/>
       <c r="AH48" s="55"/>
     </row>
-    <row r="49" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B49" s="43"/>
       <c r="C49" s="44" t="str">
         <f>IF(ISBLANK(B49),"",VLOOKUP(B49,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5132,7 +5138,7 @@
       <c r="AG49" s="54"/>
       <c r="AH49" s="55"/>
     </row>
-    <row r="50" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B50" s="43"/>
       <c r="C50" s="44" t="str">
         <f>IF(ISBLANK(B50),"",VLOOKUP(B50,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5170,7 +5176,7 @@
       <c r="AG50" s="54"/>
       <c r="AH50" s="55"/>
     </row>
-    <row r="51" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B51" s="43"/>
       <c r="C51" s="44" t="str">
         <f>IF(ISBLANK(B51),"",VLOOKUP(B51,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5208,7 +5214,7 @@
       <c r="AG51" s="54"/>
       <c r="AH51" s="55"/>
     </row>
-    <row r="52" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B52" s="43"/>
       <c r="C52" s="44" t="str">
         <f>IF(ISBLANK(B52),"",VLOOKUP(B52,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5246,7 +5252,7 @@
       <c r="AG52" s="54"/>
       <c r="AH52" s="55"/>
     </row>
-    <row r="53" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B53" s="43"/>
       <c r="C53" s="44" t="str">
         <f>IF(ISBLANK(B53),"",VLOOKUP(B53,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5284,7 +5290,7 @@
       <c r="AG53" s="54"/>
       <c r="AH53" s="55"/>
     </row>
-    <row r="54" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B54" s="43"/>
       <c r="C54" s="44" t="str">
         <f>IF(ISBLANK(B54),"",VLOOKUP(B54,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5322,7 +5328,7 @@
       <c r="AG54" s="54"/>
       <c r="AH54" s="55"/>
     </row>
-    <row r="55" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B55" s="43"/>
       <c r="C55" s="44" t="str">
         <f>IF(ISBLANK(B55),"",VLOOKUP(B55,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5360,7 +5366,7 @@
       <c r="AG55" s="54"/>
       <c r="AH55" s="55"/>
     </row>
-    <row r="56" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B56" s="43"/>
       <c r="C56" s="44" t="str">
         <f>IF(ISBLANK(B56),"",VLOOKUP(B56,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5398,7 +5404,7 @@
       <c r="AG56" s="54"/>
       <c r="AH56" s="55"/>
     </row>
-    <row r="57" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B57" s="43"/>
       <c r="C57" s="44" t="str">
         <f>IF(ISBLANK(B57),"",VLOOKUP(B57,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5436,7 +5442,7 @@
       <c r="AG57" s="54"/>
       <c r="AH57" s="55"/>
     </row>
-    <row r="58" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B58" s="43"/>
       <c r="C58" s="44" t="str">
         <f>IF(ISBLANK(B58),"",VLOOKUP(B58,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5474,7 +5480,7 @@
       <c r="AG58" s="54"/>
       <c r="AH58" s="55"/>
     </row>
-    <row r="59" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B59" s="43"/>
       <c r="C59" s="44" t="str">
         <f>IF(ISBLANK(B59),"",VLOOKUP(B59,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5512,7 +5518,7 @@
       <c r="AG59" s="54"/>
       <c r="AH59" s="55"/>
     </row>
-    <row r="60" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B60" s="43"/>
       <c r="C60" s="44" t="str">
         <f>IF(ISBLANK(B60),"",VLOOKUP(B60,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5550,7 +5556,7 @@
       <c r="AG60" s="54"/>
       <c r="AH60" s="55"/>
     </row>
-    <row r="61" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B61" s="43"/>
       <c r="C61" s="44" t="str">
         <f>IF(ISBLANK(B61),"",VLOOKUP(B61,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5588,7 +5594,7 @@
       <c r="AG61" s="54"/>
       <c r="AH61" s="55"/>
     </row>
-    <row r="62" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B62" s="43"/>
       <c r="C62" s="44" t="str">
         <f>IF(ISBLANK(B62),"",VLOOKUP(B62,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5626,7 +5632,7 @@
       <c r="AG62" s="54"/>
       <c r="AH62" s="55"/>
     </row>
-    <row r="63" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B63" s="43"/>
       <c r="C63" s="44" t="str">
         <f>IF(ISBLANK(B63),"",VLOOKUP(B63,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5664,7 +5670,7 @@
       <c r="AG63" s="54"/>
       <c r="AH63" s="55"/>
     </row>
-    <row r="64" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B64" s="43"/>
       <c r="C64" s="44" t="str">
         <f>IF(ISBLANK(B64),"",VLOOKUP(B64,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5702,7 +5708,7 @@
       <c r="AG64" s="54"/>
       <c r="AH64" s="55"/>
     </row>
-    <row r="65" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B65" s="43"/>
       <c r="C65" s="44" t="str">
         <f>IF(ISBLANK(B65),"",VLOOKUP(B65,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5740,7 +5746,7 @@
       <c r="AG65" s="54"/>
       <c r="AH65" s="55"/>
     </row>
-    <row r="66" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B66" s="43"/>
       <c r="C66" s="44" t="str">
         <f>IF(ISBLANK(B66),"",VLOOKUP(B66,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5778,7 +5784,7 @@
       <c r="AG66" s="54"/>
       <c r="AH66" s="55"/>
     </row>
-    <row r="67" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B67" s="43"/>
       <c r="C67" s="44" t="str">
         <f>IF(ISBLANK(B67),"",VLOOKUP(B67,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5816,7 +5822,7 @@
       <c r="AG67" s="54"/>
       <c r="AH67" s="55"/>
     </row>
-    <row r="68" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B68" s="43"/>
       <c r="C68" s="44" t="str">
         <f>IF(ISBLANK(B68),"",VLOOKUP(B68,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5854,7 +5860,7 @@
       <c r="AG68" s="54"/>
       <c r="AH68" s="55"/>
     </row>
-    <row r="69" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B69" s="43"/>
       <c r="C69" s="44" t="str">
         <f>IF(ISBLANK(B69),"",VLOOKUP(B69,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5892,7 +5898,7 @@
       <c r="AG69" s="54"/>
       <c r="AH69" s="55"/>
     </row>
-    <row r="70" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B70" s="43"/>
       <c r="C70" s="44" t="str">
         <f>IF(ISBLANK(B70),"",VLOOKUP(B70,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5930,7 +5936,7 @@
       <c r="AG70" s="54"/>
       <c r="AH70" s="55"/>
     </row>
-    <row r="71" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B71" s="43"/>
       <c r="C71" s="44" t="str">
         <f>IF(ISBLANK(B71),"",VLOOKUP(B71,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -5968,7 +5974,7 @@
       <c r="AG71" s="54"/>
       <c r="AH71" s="55"/>
     </row>
-    <row r="72" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B72" s="43"/>
       <c r="C72" s="44" t="str">
         <f>IF(ISBLANK(B72),"",VLOOKUP(B72,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6006,7 +6012,7 @@
       <c r="AG72" s="54"/>
       <c r="AH72" s="55"/>
     </row>
-    <row r="73" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B73" s="43"/>
       <c r="C73" s="44" t="str">
         <f>IF(ISBLANK(B73),"",VLOOKUP(B73,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6044,7 +6050,7 @@
       <c r="AG73" s="54"/>
       <c r="AH73" s="55"/>
     </row>
-    <row r="74" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B74" s="43"/>
       <c r="C74" s="44" t="str">
         <f>IF(ISBLANK(B74),"",VLOOKUP(B74,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6082,7 +6088,7 @@
       <c r="AG74" s="54"/>
       <c r="AH74" s="55"/>
     </row>
-    <row r="75" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B75" s="43"/>
       <c r="C75" s="44" t="str">
         <f>IF(ISBLANK(B75),"",VLOOKUP(B75,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6120,7 +6126,7 @@
       <c r="AG75" s="54"/>
       <c r="AH75" s="55"/>
     </row>
-    <row r="76" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B76" s="43"/>
       <c r="C76" s="44" t="str">
         <f>IF(ISBLANK(B76),"",VLOOKUP(B76,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6158,7 +6164,7 @@
       <c r="AG76" s="54"/>
       <c r="AH76" s="55"/>
     </row>
-    <row r="77" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B77" s="43"/>
       <c r="C77" s="44" t="str">
         <f>IF(ISBLANK(B77),"",VLOOKUP(B77,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6196,7 +6202,7 @@
       <c r="AG77" s="54"/>
       <c r="AH77" s="55"/>
     </row>
-    <row r="78" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B78" s="43"/>
       <c r="C78" s="44" t="str">
         <f>IF(ISBLANK(B78),"",VLOOKUP(B78,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6234,7 +6240,7 @@
       <c r="AG78" s="54"/>
       <c r="AH78" s="55"/>
     </row>
-    <row r="79" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B79" s="43"/>
       <c r="C79" s="44" t="str">
         <f>IF(ISBLANK(B79),"",VLOOKUP(B79,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6272,7 +6278,7 @@
       <c r="AG79" s="54"/>
       <c r="AH79" s="55"/>
     </row>
-    <row r="80" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B80" s="43"/>
       <c r="C80" s="44" t="str">
         <f>IF(ISBLANK(B80),"",VLOOKUP(B80,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6310,7 +6316,7 @@
       <c r="AG80" s="54"/>
       <c r="AH80" s="55"/>
     </row>
-    <row r="81" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B81" s="43"/>
       <c r="C81" s="44" t="str">
         <f>IF(ISBLANK(B81),"",VLOOKUP(B81,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6348,7 +6354,7 @@
       <c r="AG81" s="54"/>
       <c r="AH81" s="55"/>
     </row>
-    <row r="82" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B82" s="43"/>
       <c r="C82" s="44" t="str">
         <f>IF(ISBLANK(B82),"",VLOOKUP(B82,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6386,7 +6392,7 @@
       <c r="AG82" s="54"/>
       <c r="AH82" s="55"/>
     </row>
-    <row r="83" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B83" s="43"/>
       <c r="C83" s="44" t="str">
         <f>IF(ISBLANK(B83),"",VLOOKUP(B83,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6424,7 +6430,7 @@
       <c r="AG83" s="54"/>
       <c r="AH83" s="55"/>
     </row>
-    <row r="84" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B84" s="43"/>
       <c r="C84" s="44" t="str">
         <f>IF(ISBLANK(B84),"",VLOOKUP(B84,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6462,7 +6468,7 @@
       <c r="AG84" s="54"/>
       <c r="AH84" s="55"/>
     </row>
-    <row r="85" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B85" s="43"/>
       <c r="C85" s="44" t="str">
         <f>IF(ISBLANK(B85),"",VLOOKUP(B85,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6500,7 +6506,7 @@
       <c r="AG85" s="54"/>
       <c r="AH85" s="55"/>
     </row>
-    <row r="86" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B86" s="43"/>
       <c r="C86" s="44" t="str">
         <f>IF(ISBLANK(B86),"",VLOOKUP(B86,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6538,7 +6544,7 @@
       <c r="AG86" s="54"/>
       <c r="AH86" s="55"/>
     </row>
-    <row r="87" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B87" s="43"/>
       <c r="C87" s="44" t="str">
         <f>IF(ISBLANK(B87),"",VLOOKUP(B87,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6576,7 +6582,7 @@
       <c r="AG87" s="54"/>
       <c r="AH87" s="55"/>
     </row>
-    <row r="88" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B88" s="43"/>
       <c r="C88" s="44" t="str">
         <f>IF(ISBLANK(B88),"",VLOOKUP(B88,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6614,7 +6620,7 @@
       <c r="AG88" s="54"/>
       <c r="AH88" s="55"/>
     </row>
-    <row r="89" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B89" s="43"/>
       <c r="C89" s="44" t="str">
         <f>IF(ISBLANK(B89),"",VLOOKUP(B89,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6652,7 +6658,7 @@
       <c r="AG89" s="54"/>
       <c r="AH89" s="55"/>
     </row>
-    <row r="90" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B90" s="43"/>
       <c r="C90" s="44" t="str">
         <f>IF(ISBLANK(B90),"",VLOOKUP(B90,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6690,7 +6696,7 @@
       <c r="AG90" s="54"/>
       <c r="AH90" s="55"/>
     </row>
-    <row r="91" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B91" s="43"/>
       <c r="C91" s="44" t="str">
         <f>IF(ISBLANK(B91),"",VLOOKUP(B91,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6728,7 +6734,7 @@
       <c r="AG91" s="54"/>
       <c r="AH91" s="55"/>
     </row>
-    <row r="92" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B92" s="43"/>
       <c r="C92" s="44" t="str">
         <f>IF(ISBLANK(B92),"",VLOOKUP(B92,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6766,7 +6772,7 @@
       <c r="AG92" s="54"/>
       <c r="AH92" s="55"/>
     </row>
-    <row r="93" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B93" s="43"/>
       <c r="C93" s="44" t="str">
         <f>IF(ISBLANK(B93),"",VLOOKUP(B93,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6804,7 +6810,7 @@
       <c r="AG93" s="54"/>
       <c r="AH93" s="55"/>
     </row>
-    <row r="94" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B94" s="43"/>
       <c r="C94" s="44" t="str">
         <f>IF(ISBLANK(B94),"",VLOOKUP(B94,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6842,7 +6848,7 @@
       <c r="AG94" s="54"/>
       <c r="AH94" s="55"/>
     </row>
-    <row r="95" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B95" s="43"/>
       <c r="C95" s="44" t="str">
         <f>IF(ISBLANK(B95),"",VLOOKUP(B95,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6880,7 +6886,7 @@
       <c r="AG95" s="54"/>
       <c r="AH95" s="55"/>
     </row>
-    <row r="96" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B96" s="43"/>
       <c r="C96" s="44" t="str">
         <f>IF(ISBLANK(B96),"",VLOOKUP(B96,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6918,7 +6924,7 @@
       <c r="AG96" s="54"/>
       <c r="AH96" s="55"/>
     </row>
-    <row r="97" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B97" s="43"/>
       <c r="C97" s="44" t="str">
         <f>IF(ISBLANK(B97),"",VLOOKUP(B97,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6956,7 +6962,7 @@
       <c r="AG97" s="54"/>
       <c r="AH97" s="55"/>
     </row>
-    <row r="98" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B98" s="43"/>
       <c r="C98" s="44" t="str">
         <f>IF(ISBLANK(B98),"",VLOOKUP(B98,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -6994,7 +7000,7 @@
       <c r="AG98" s="54"/>
       <c r="AH98" s="55"/>
     </row>
-    <row r="99" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B99" s="43"/>
       <c r="C99" s="44" t="str">
         <f>IF(ISBLANK(B99),"",VLOOKUP(B99,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7032,7 +7038,7 @@
       <c r="AG99" s="54"/>
       <c r="AH99" s="55"/>
     </row>
-    <row r="100" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B100" s="43"/>
       <c r="C100" s="44" t="str">
         <f>IF(ISBLANK(B100),"",VLOOKUP(B100,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7070,7 +7076,7 @@
       <c r="AG100" s="54"/>
       <c r="AH100" s="55"/>
     </row>
-    <row r="101" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B101" s="43"/>
       <c r="C101" s="44" t="str">
         <f>IF(ISBLANK(B101),"",VLOOKUP(B101,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7108,7 +7114,7 @@
       <c r="AG101" s="54"/>
       <c r="AH101" s="55"/>
     </row>
-    <row r="102" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B102" s="43"/>
       <c r="C102" s="44" t="str">
         <f>IF(ISBLANK(B102),"",VLOOKUP(B102,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7146,7 +7152,7 @@
       <c r="AG102" s="54"/>
       <c r="AH102" s="55"/>
     </row>
-    <row r="103" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B103" s="43"/>
       <c r="C103" s="44" t="str">
         <f>IF(ISBLANK(B103),"",VLOOKUP(B103,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7184,7 +7190,7 @@
       <c r="AG103" s="54"/>
       <c r="AH103" s="55"/>
     </row>
-    <row r="104" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B104" s="43"/>
       <c r="C104" s="44" t="str">
         <f>IF(ISBLANK(B104),"",VLOOKUP(B104,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7222,7 +7228,7 @@
       <c r="AG104" s="54"/>
       <c r="AH104" s="55"/>
     </row>
-    <row r="105" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B105" s="43"/>
       <c r="C105" s="44" t="str">
         <f>IF(ISBLANK(B105),"",VLOOKUP(B105,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7260,7 +7266,7 @@
       <c r="AG105" s="54"/>
       <c r="AH105" s="55"/>
     </row>
-    <row r="106" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B106" s="43"/>
       <c r="C106" s="44" t="str">
         <f>IF(ISBLANK(B106),"",VLOOKUP(B106,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7298,7 +7304,7 @@
       <c r="AG106" s="54"/>
       <c r="AH106" s="55"/>
     </row>
-    <row r="107" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B107" s="43"/>
       <c r="C107" s="44" t="str">
         <f>IF(ISBLANK(B107),"",VLOOKUP(B107,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7336,7 +7342,7 @@
       <c r="AG107" s="54"/>
       <c r="AH107" s="55"/>
     </row>
-    <row r="108" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B108" s="43"/>
       <c r="C108" s="44" t="str">
         <f>IF(ISBLANK(B108),"",VLOOKUP(B108,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7374,7 +7380,7 @@
       <c r="AG108" s="54"/>
       <c r="AH108" s="55"/>
     </row>
-    <row r="109" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B109" s="43"/>
       <c r="C109" s="44" t="str">
         <f>IF(ISBLANK(B109),"",VLOOKUP(B109,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7412,7 +7418,7 @@
       <c r="AG109" s="54"/>
       <c r="AH109" s="55"/>
     </row>
-    <row r="110" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B110" s="43"/>
       <c r="C110" s="44" t="str">
         <f>IF(ISBLANK(B110),"",VLOOKUP(B110,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7450,7 +7456,7 @@
       <c r="AG110" s="54"/>
       <c r="AH110" s="55"/>
     </row>
-    <row r="111" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B111" s="43"/>
       <c r="C111" s="44" t="str">
         <f>IF(ISBLANK(B111),"",VLOOKUP(B111,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7488,7 +7494,7 @@
       <c r="AG111" s="54"/>
       <c r="AH111" s="55"/>
     </row>
-    <row r="112" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B112" s="43"/>
       <c r="C112" s="44" t="str">
         <f>IF(ISBLANK(B112),"",VLOOKUP(B112,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7526,7 +7532,7 @@
       <c r="AG112" s="54"/>
       <c r="AH112" s="55"/>
     </row>
-    <row r="113" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B113" s="43"/>
       <c r="C113" s="44" t="str">
         <f>IF(ISBLANK(B113),"",VLOOKUP(B113,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7564,7 +7570,7 @@
       <c r="AG113" s="54"/>
       <c r="AH113" s="55"/>
     </row>
-    <row r="114" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B114" s="43"/>
       <c r="C114" s="44" t="str">
         <f>IF(ISBLANK(B114),"",VLOOKUP(B114,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7602,7 +7608,7 @@
       <c r="AG114" s="54"/>
       <c r="AH114" s="55"/>
     </row>
-    <row r="115" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B115" s="43"/>
       <c r="C115" s="44" t="str">
         <f>IF(ISBLANK(B115),"",VLOOKUP(B115,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7640,7 +7646,7 @@
       <c r="AG115" s="54"/>
       <c r="AH115" s="55"/>
     </row>
-    <row r="116" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B116" s="43"/>
       <c r="C116" s="44" t="str">
         <f>IF(ISBLANK(B116),"",VLOOKUP(B116,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7678,7 +7684,7 @@
       <c r="AG116" s="54"/>
       <c r="AH116" s="55"/>
     </row>
-    <row r="117" spans="2:34" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B117" s="43"/>
       <c r="C117" s="44" t="str">
         <f>IF(ISBLANK(B117),"",VLOOKUP(B117,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7716,7 +7722,7 @@
       <c r="AG117" s="54"/>
       <c r="AH117" s="55"/>
     </row>
-    <row r="118" spans="2:34" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="118" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B118" s="45"/>
       <c r="C118" s="46" t="str">
         <f>IF(ISBLANK(B118),"",VLOOKUP(B118,'Codes projet'!$A$2:$B$802,2,FALSE))</f>
@@ -7754,7 +7760,7 @@
       <c r="AG118" s="57"/>
       <c r="AH118" s="58"/>
     </row>
-    <row r="119" spans="2:34" s="34" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:34" s="34" customFormat="1" x14ac:dyDescent="0.25">
       <c r="D119" s="60" t="str">
         <f>IF(D133&lt;&gt;D134,IF(D133&gt;D134,TEXT(D133-D134,"-HH::MM"),TEXT(D134-D133,"HH::MM")),"")</f>
         <v/>
@@ -7880,7 +7886,7 @@
         <v>-08:00</v>
       </c>
     </row>
-    <row r="120" spans="2:34" s="34" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:34" s="34" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D120" s="60"/>
       <c r="E120" s="60"/>
       <c r="F120" s="60"/>
@@ -7913,7 +7919,7 @@
       <c r="AG120" s="60"/>
       <c r="AH120" s="60"/>
     </row>
-    <row r="121" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D121" s="60"/>
       <c r="E121" s="60"/>
       <c r="F121" s="60"/>
@@ -7946,7 +7952,7 @@
       <c r="AG121" s="60"/>
       <c r="AH121" s="60"/>
     </row>
-    <row r="122" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D122" s="60"/>
       <c r="E122" s="60"/>
       <c r="F122" s="60"/>
@@ -7979,7 +7985,7 @@
       <c r="AG122" s="60"/>
       <c r="AH122" s="60"/>
     </row>
-    <row r="123" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D123" s="60"/>
       <c r="E123" s="60"/>
       <c r="F123" s="60"/>
@@ -8012,7 +8018,7 @@
       <c r="AG123" s="60"/>
       <c r="AH123" s="60"/>
     </row>
-    <row r="124" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D124" s="60"/>
       <c r="E124" s="60"/>
       <c r="F124" s="60"/>
@@ -8045,7 +8051,7 @@
       <c r="AG124" s="60"/>
       <c r="AH124" s="60"/>
     </row>
-    <row r="125" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D125" s="60"/>
       <c r="E125" s="60"/>
       <c r="F125" s="60"/>
@@ -8078,7 +8084,7 @@
       <c r="AG125" s="60"/>
       <c r="AH125" s="60"/>
     </row>
-    <row r="126" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D126" s="60"/>
       <c r="E126" s="60"/>
       <c r="F126" s="60"/>
@@ -8111,7 +8117,7 @@
       <c r="AG126" s="60"/>
       <c r="AH126" s="60"/>
     </row>
-    <row r="127" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D127" s="60"/>
       <c r="E127" s="60"/>
       <c r="F127" s="60"/>
@@ -8144,7 +8150,7 @@
       <c r="AG127" s="60"/>
       <c r="AH127" s="60"/>
     </row>
-    <row r="128" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="D128" s="60"/>
       <c r="E128" s="60"/>
       <c r="F128" s="60"/>
@@ -8177,7 +8183,7 @@
       <c r="AG128" s="60"/>
       <c r="AH128" s="60"/>
     </row>
-    <row r="131" spans="2:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="2:34" hidden="1" x14ac:dyDescent="0.25">
       <c r="C131" t="s">
         <v>25</v>
       </c>
@@ -8194,7 +8200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="2:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="2:34" hidden="1" x14ac:dyDescent="0.25">
       <c r="C132" t="s">
         <v>26</v>
       </c>
@@ -8323,7 +8329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B133" s="3"/>
       <c r="C133" s="34" t="s">
         <v>27</v>
@@ -8453,7 +8459,7 @@
         <v>0.33333333333333337</v>
       </c>
     </row>
-    <row r="134" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="C134" s="34" t="s">
         <v>28</v>
       </c>
@@ -8582,7 +8588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="2:34" s="34" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="C135" s="34" t="s">
         <v>29</v>
       </c>
@@ -8711,7 +8717,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="2:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="2:34" hidden="1" x14ac:dyDescent="0.25">
       <c r="C137" s="34" t="s">
         <v>30</v>
       </c>
@@ -8840,7 +8846,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="2:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="2:34" hidden="1" x14ac:dyDescent="0.25">
       <c r="C138" s="34" t="s">
         <v>31</v>
       </c>
@@ -8969,7 +8975,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="2:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:34" hidden="1" x14ac:dyDescent="0.25">
       <c r="C139" s="34" t="s">
         <v>23</v>
       </c>
@@ -9098,7 +9104,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="2:34" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="2:34" hidden="1" x14ac:dyDescent="0.25">
       <c r="C140" s="34" t="s">
         <v>32</v>
       </c>
@@ -9261,24 +9267,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8185E767-BB80-4F39-AD8C-03A0BD11B651}">
   <dimension ref="A1:S50"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.54296875" style="12" customWidth="1"/>
-    <col min="2" max="2" width="3.54296875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" style="12" customWidth="1"/>
-    <col min="4" max="4" width="8.26953125" style="12" customWidth="1"/>
-    <col min="5" max="5" width="1.7265625" style="12" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" style="12" customWidth="1"/>
-    <col min="7" max="7" width="1.7265625" style="12" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" style="12" customWidth="1"/>
+    <col min="2" max="2" width="3.5703125" style="12" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" style="12" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" style="12" customWidth="1"/>
+    <col min="5" max="5" width="1.7109375" style="12" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" style="12" customWidth="1"/>
+    <col min="7" max="7" width="1.7109375" style="12" customWidth="1"/>
     <col min="8" max="8" width="13" style="12" customWidth="1"/>
-    <col min="9" max="9" width="7.26953125" style="12" customWidth="1"/>
-    <col min="10" max="10" width="21.54296875" style="12" customWidth="1"/>
-    <col min="11" max="11" width="3.54296875" style="12" customWidth="1"/>
+    <col min="9" max="9" width="7.28515625" style="12" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" style="12" customWidth="1"/>
+    <col min="11" max="11" width="3.5703125" style="12" customWidth="1"/>
     <col min="12" max="12" width="3" style="12" customWidth="1"/>
-    <col min="13" max="16384" width="9.1796875" style="12" hidden="1"/>
+    <col min="13" max="16384" width="9.140625" style="12" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="B1" s="13"/>
       <c r="C1" s="13"/>
       <c r="D1" s="13"/>
@@ -9290,7 +9296,7 @@
       <c r="J1" s="13"/>
       <c r="K1" s="13"/>
     </row>
-    <row r="2" spans="1:19" ht="36.75" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:19" ht="36.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="14"/>
       <c r="B2" s="15"/>
       <c r="C2" s="16"/>
@@ -9306,7 +9312,7 @@
       <c r="K2" s="142"/>
       <c r="L2" s="17"/>
     </row>
-    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="14"/>
       <c r="B3" s="18"/>
       <c r="C3" s="19"/>
@@ -9323,7 +9329,7 @@
       <c r="K3" s="144"/>
       <c r="L3" s="20"/>
     </row>
-    <row r="4" spans="1:19" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14"/>
       <c r="B4" s="7"/>
       <c r="C4" s="30" t="s">
@@ -9347,7 +9353,7 @@
       <c r="K4" s="8"/>
       <c r="L4" s="20"/>
     </row>
-    <row r="5" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23"/>
       <c r="B5" s="24"/>
       <c r="C5" s="25" t="s">
@@ -9367,7 +9373,7 @@
       <c r="K5" s="27"/>
       <c r="L5" s="28"/>
     </row>
-    <row r="6" spans="1:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="23"/>
       <c r="B6" s="28"/>
       <c r="C6" s="69"/>
@@ -9381,7 +9387,7 @@
       <c r="K6" s="23"/>
       <c r="L6" s="28"/>
     </row>
-    <row r="7" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14"/>
       <c r="B7" s="7"/>
       <c r="C7" s="1">
@@ -9421,7 +9427,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="14"/>
       <c r="B8" s="9"/>
       <c r="C8" s="1">
@@ -9459,7 +9465,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="14"/>
       <c r="B9" s="9"/>
       <c r="C9" s="1">
@@ -9497,7 +9503,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="14"/>
       <c r="B10" s="9"/>
       <c r="C10" s="1">
@@ -9535,7 +9541,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14"/>
       <c r="B11" s="9"/>
       <c r="C11" s="1">
@@ -9573,7 +9579,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14"/>
       <c r="B12" s="9"/>
       <c r="C12" s="1">
@@ -9611,7 +9617,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="14"/>
       <c r="B13" s="9"/>
       <c r="C13" s="1">
@@ -9649,7 +9655,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="14"/>
       <c r="B14" s="9"/>
       <c r="C14" s="1">
@@ -9687,7 +9693,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="14"/>
       <c r="B15" s="9"/>
       <c r="C15" s="1">
@@ -9725,7 +9731,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="14"/>
       <c r="B16" s="9"/>
       <c r="C16" s="1">
@@ -9763,7 +9769,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="14"/>
       <c r="B17" s="9"/>
       <c r="C17" s="1">
@@ -9801,7 +9807,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="14"/>
       <c r="B18" s="9"/>
       <c r="C18" s="1">
@@ -9839,7 +9845,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="14"/>
       <c r="B19" s="9"/>
       <c r="C19" s="1">
@@ -9877,7 +9883,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="14"/>
       <c r="B20" s="9"/>
       <c r="C20" s="1">
@@ -9915,7 +9921,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="14"/>
       <c r="B21" s="9"/>
       <c r="C21" s="1">
@@ -9953,7 +9959,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="14"/>
       <c r="B22" s="7"/>
       <c r="C22" s="1">
@@ -9991,7 +9997,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="14"/>
       <c r="B23" s="7"/>
       <c r="C23" s="1">
@@ -10029,7 +10035,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="14"/>
       <c r="B24" s="7"/>
       <c r="C24" s="1">
@@ -10067,7 +10073,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="14"/>
       <c r="B25" s="9"/>
       <c r="C25" s="1">
@@ -10105,7 +10111,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="14"/>
       <c r="B26" s="7"/>
       <c r="C26" s="1">
@@ -10143,7 +10149,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="14"/>
       <c r="B27" s="7"/>
       <c r="C27" s="1">
@@ -10181,7 +10187,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="14"/>
       <c r="B28" s="7"/>
       <c r="C28" s="1">
@@ -10219,7 +10225,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="14"/>
       <c r="B29" s="7"/>
       <c r="C29" s="1">
@@ -10257,7 +10263,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="14"/>
       <c r="B30" s="7"/>
       <c r="C30" s="1">
@@ -10295,7 +10301,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="7"/>
       <c r="C31" s="1">
@@ -10333,7 +10339,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="14"/>
       <c r="B32" s="7"/>
       <c r="C32" s="1">
@@ -10371,7 +10377,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="14"/>
       <c r="B33" s="7"/>
       <c r="C33" s="1">
@@ -10409,7 +10415,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="14"/>
       <c r="B34" s="7"/>
       <c r="C34" s="1">
@@ -10447,7 +10453,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="14"/>
       <c r="B35" s="7"/>
       <c r="C35" s="1">
@@ -10485,7 +10491,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="14"/>
       <c r="B36" s="7"/>
       <c r="C36" s="1">
@@ -10523,7 +10529,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:19" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="14"/>
       <c r="B37" s="7"/>
       <c r="C37" s="1">
@@ -10561,7 +10567,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:19" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14"/>
       <c r="B38" s="10"/>
       <c r="C38" s="2"/>
@@ -10575,7 +10581,7 @@
       <c r="K38" s="11"/>
       <c r="L38" s="20"/>
     </row>
-    <row r="39" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="14"/>
       <c r="B39" s="15"/>
       <c r="C39" s="16"/>
@@ -10589,7 +10595,7 @@
       <c r="K39" s="21"/>
       <c r="L39" s="20"/>
     </row>
-    <row r="40" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:19" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="8"/>
       <c r="B40" s="7"/>
       <c r="D40" s="154">
@@ -10607,7 +10613,7 @@
       <c r="K40" s="8"/>
       <c r="L40" s="7"/>
     </row>
-    <row r="41" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:19" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="14"/>
       <c r="B41" s="18"/>
       <c r="C41" s="13"/>
@@ -10621,7 +10627,7 @@
       <c r="K41" s="22"/>
       <c r="L41" s="20"/>
     </row>
-    <row r="42" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:19" ht="9.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
       <c r="C42" s="16"/>
@@ -10635,7 +10641,7 @@
       <c r="K42" s="21"/>
       <c r="L42" s="20"/>
     </row>
-    <row r="43" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="14"/>
       <c r="B43" s="20"/>
       <c r="C43" s="145" t="s">
@@ -10650,7 +10656,7 @@
       <c r="K43" s="31"/>
       <c r="L43" s="20"/>
     </row>
-    <row r="44" spans="1:19" ht="16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="14"/>
       <c r="B44" s="20"/>
       <c r="C44" s="151"/>
@@ -10666,7 +10672,7 @@
       <c r="K44" s="32"/>
       <c r="L44" s="20"/>
     </row>
-    <row r="45" spans="1:19" ht="15" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:19" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="14"/>
       <c r="B45" s="20"/>
       <c r="C45" s="151"/>
@@ -10682,7 +10688,7 @@
       <c r="K45" s="33"/>
       <c r="L45" s="20"/>
     </row>
-    <row r="46" spans="1:19" ht="55.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:19" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
       <c r="B46" s="20"/>
       <c r="C46" s="151"/>
@@ -10698,7 +10704,7 @@
       <c r="K46" s="33"/>
       <c r="L46" s="20"/>
     </row>
-    <row r="47" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A47" s="14"/>
       <c r="B47" s="18"/>
       <c r="C47" s="13"/>
@@ -10712,7 +10718,7 @@
       <c r="K47" s="22"/>
       <c r="L47" s="20"/>
     </row>
-    <row r="48" spans="1:19" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="B48" s="16"/>
       <c r="C48" s="16"/>
       <c r="D48" s="16"/>
@@ -10724,8 +10730,8 @@
       <c r="J48" s="16"/>
       <c r="K48" s="16"/>
     </row>
-    <row r="49" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="50" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="49" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="50" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="43">
     <mergeCell ref="C44:F46"/>
@@ -10792,26 +10798,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCD68CF1-8051-41F5-B1AE-36E45401E4F1}">
   <dimension ref="B1:N140"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.1796875" style="34" customWidth="1"/>
-    <col min="2" max="2" width="11.54296875" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.81640625" style="34" customWidth="1"/>
-    <col min="4" max="4" width="10.81640625" style="34" customWidth="1"/>
-    <col min="5" max="5" width="10.7265625" style="34" customWidth="1"/>
-    <col min="6" max="6" width="16.26953125" style="34" customWidth="1"/>
-    <col min="7" max="7" width="9.26953125" style="34" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" style="34" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" style="34" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" style="34" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="34" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" style="34" customWidth="1"/>
+    <col min="7" max="7" width="9.28515625" style="34" customWidth="1"/>
     <col min="8" max="8" width="4" style="34" customWidth="1"/>
-    <col min="9" max="10" width="9.1796875" style="34" hidden="1"/>
-    <col min="11" max="11" width="5.453125" style="34" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="10.26953125" style="34" hidden="1" customWidth="1"/>
-    <col min="13" max="13" width="9.1796875" style="34" hidden="1"/>
-    <col min="14" max="14" width="1.453125" style="34" hidden="1" customWidth="1"/>
+    <col min="9" max="10" width="9.140625" style="34" hidden="1"/>
+    <col min="11" max="11" width="5.42578125" style="34" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="10.28515625" style="34" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" style="34" hidden="1"/>
+    <col min="14" max="14" width="1.42578125" style="34" hidden="1" customWidth="1"/>
     <col min="15" max="16384" width="0" style="34" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:12" ht="26" x14ac:dyDescent="0.6">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:12" ht="26.25" x14ac:dyDescent="0.4">
       <c r="B2" s="167">
         <f>Configuration!D13</f>
         <v>0</v>
@@ -10822,8 +10828,8 @@
       <c r="F2" s="168"/>
       <c r="G2" s="169"/>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="2:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B4" s="76" t="s">
         <v>11</v>
       </c>
@@ -10836,7 +10842,7 @@
       <c r="F4" s="78"/>
       <c r="G4" s="79"/>
     </row>
-    <row r="5" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="80" t="s">
         <v>12</v>
       </c>
@@ -10846,7 +10852,7 @@
       </c>
       <c r="G5" s="82"/>
     </row>
-    <row r="6" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B6" s="80" t="s">
         <v>13</v>
       </c>
@@ -10860,7 +10866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B7" s="80" t="s">
         <v>14</v>
       </c>
@@ -10870,7 +10876,7 @@
       </c>
       <c r="G7" s="85"/>
     </row>
-    <row r="8" spans="2:12" ht="18.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B8" s="86" t="s">
         <v>45</v>
       </c>
@@ -10883,12 +10889,12 @@
       <c r="F8" s="88"/>
       <c r="G8" s="89"/>
     </row>
-    <row r="9" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C9" s="71"/>
       <c r="D9" s="71"/>
     </row>
-    <row r="10" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="11" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E11" s="72" t="s">
         <v>37</v>
       </c>
@@ -10905,7 +10911,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="90"/>
       <c r="C12" s="128" t="s">
         <v>49</v>
@@ -10932,7 +10938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="104" t="str">
         <f>IF(ISBLANK(Prestations!B7),"",Prestations!B7)</f>
         <v/>
@@ -10963,7 +10969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B8),"",Prestations!B8)</f>
         <v/>
@@ -10994,7 +11000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B9),"",Prestations!B9)</f>
         <v/>
@@ -11025,7 +11031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B10),"",Prestations!B10)</f>
         <v/>
@@ -11056,7 +11062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B11),"",Prestations!B11)</f>
         <v/>
@@ -11087,7 +11093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B12),"",Prestations!B12)</f>
         <v/>
@@ -11118,7 +11124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B13),"",Prestations!B13)</f>
         <v/>
@@ -11149,7 +11155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B14),"",Prestations!B14)</f>
         <v/>
@@ -11180,7 +11186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B15),"",Prestations!B15)</f>
         <v/>
@@ -11211,7 +11217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B16),"",Prestations!B16)</f>
         <v/>
@@ -11242,7 +11248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B17),"",Prestations!B17)</f>
         <v/>
@@ -11273,7 +11279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B18),"",Prestations!B18)</f>
         <v/>
@@ -11304,7 +11310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B19),"",Prestations!B19)</f>
         <v/>
@@ -11335,7 +11341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B20),"",Prestations!B20)</f>
         <v/>
@@ -11366,7 +11372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B21),"",Prestations!B21)</f>
         <v/>
@@ -11397,7 +11403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B22),"",Prestations!B22)</f>
         <v/>
@@ -11428,7 +11434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B23),"",Prestations!B23)</f>
         <v/>
@@ -11459,7 +11465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B24),"",Prestations!B24)</f>
         <v/>
@@ -11490,7 +11496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B25),"",Prestations!B25)</f>
         <v/>
@@ -11521,7 +11527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B26),"",Prestations!B26)</f>
         <v/>
@@ -11552,7 +11558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B33" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B27),"",Prestations!B27)</f>
         <v/>
@@ -11583,7 +11589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B28),"",Prestations!B28)</f>
         <v/>
@@ -11614,7 +11620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B35" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B29),"",Prestations!B29)</f>
         <v/>
@@ -11645,7 +11651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B36" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B30),"",Prestations!B30)</f>
         <v/>
@@ -11676,7 +11682,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B37" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B31),"",Prestations!B31)</f>
         <v/>
@@ -11707,7 +11713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B32),"",Prestations!B32)</f>
         <v/>
@@ -11738,7 +11744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B39" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B33),"",Prestations!B33)</f>
         <v/>
@@ -11772,7 +11778,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B34),"",Prestations!B34)</f>
         <v/>
@@ -11803,7 +11809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B41" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B35),"",Prestations!B35)</f>
         <v/>
@@ -11834,7 +11840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B36),"",Prestations!B36)</f>
         <v/>
@@ -11865,7 +11871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B43" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B37),"",Prestations!B37)</f>
         <v/>
@@ -11896,7 +11902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B44" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B38),"",Prestations!B38)</f>
         <v/>
@@ -11927,7 +11933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B45" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B39),"",Prestations!B39)</f>
         <v/>
@@ -11958,7 +11964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B46" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B40),"",Prestations!B40)</f>
         <v/>
@@ -11989,7 +11995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B47" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B41),"",Prestations!B41)</f>
         <v/>
@@ -12020,7 +12026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B48" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B42),"",Prestations!B42)</f>
         <v/>
@@ -12051,7 +12057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B43),"",Prestations!B43)</f>
         <v/>
@@ -12082,7 +12088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B50" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B44),"",Prestations!B44)</f>
         <v/>
@@ -12113,7 +12119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B51" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B45),"",Prestations!B45)</f>
         <v/>
@@ -12144,7 +12150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B52" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B46),"",Prestations!B46)</f>
         <v/>
@@ -12175,7 +12181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B47),"",Prestations!B47)</f>
         <v/>
@@ -12206,7 +12212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B48),"",Prestations!B48)</f>
         <v/>
@@ -12237,7 +12243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B55" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B49),"",Prestations!B49)</f>
         <v/>
@@ -12268,7 +12274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B56" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B50),"",Prestations!B50)</f>
         <v/>
@@ -12299,7 +12305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B57" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B51),"",Prestations!B51)</f>
         <v/>
@@ -12330,7 +12336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B58" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B52),"",Prestations!B52)</f>
         <v/>
@@ -12361,7 +12367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B59" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B53),"",Prestations!B53)</f>
         <v/>
@@ -12392,7 +12398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B60" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B54),"",Prestations!B54)</f>
         <v/>
@@ -12423,7 +12429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B61" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B55),"",Prestations!B55)</f>
         <v/>
@@ -12454,7 +12460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B62" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B56),"",Prestations!B56)</f>
         <v/>
@@ -12485,7 +12491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B63" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B57),"",Prestations!B57)</f>
         <v/>
@@ -12516,7 +12522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B64" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B58),"",Prestations!B58)</f>
         <v/>
@@ -12547,7 +12553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B65" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B59),"",Prestations!B59)</f>
         <v/>
@@ -12578,7 +12584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B66" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B60),"",Prestations!B60)</f>
         <v/>
@@ -12612,7 +12618,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="67" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B67" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B61),"",Prestations!B61)</f>
         <v/>
@@ -12643,7 +12649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B68" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B62),"",Prestations!B62)</f>
         <v/>
@@ -12674,7 +12680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B69" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B63),"",Prestations!B63)</f>
         <v/>
@@ -12705,7 +12711,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B70" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B64),"",Prestations!B64)</f>
         <v/>
@@ -12736,7 +12742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B71" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B65),"",Prestations!B65)</f>
         <v/>
@@ -12767,7 +12773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B72" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B66),"",Prestations!B66)</f>
         <v/>
@@ -12798,7 +12804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B73" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B67),"",Prestations!B67)</f>
         <v/>
@@ -12829,7 +12835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B74" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B68),"",Prestations!B68)</f>
         <v/>
@@ -12860,7 +12866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B75" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B69),"",Prestations!B69)</f>
         <v/>
@@ -12891,7 +12897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B76" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B70),"",Prestations!B70)</f>
         <v/>
@@ -12922,7 +12928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B77" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B71),"",Prestations!B71)</f>
         <v/>
@@ -12953,7 +12959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="78" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B78" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B72),"",Prestations!B72)</f>
         <v/>
@@ -12984,7 +12990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B79" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B73),"",Prestations!B73)</f>
         <v/>
@@ -13015,7 +13021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B80" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B74),"",Prestations!B74)</f>
         <v/>
@@ -13046,7 +13052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="81" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B81" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B75),"",Prestations!B75)</f>
         <v/>
@@ -13077,7 +13083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="82" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B82" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B76),"",Prestations!B76)</f>
         <v/>
@@ -13108,7 +13114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="83" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B83" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B77),"",Prestations!B77)</f>
         <v/>
@@ -13139,7 +13145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="84" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B84" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B78),"",Prestations!B78)</f>
         <v/>
@@ -13170,7 +13176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="85" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B85" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B79),"",Prestations!B79)</f>
         <v/>
@@ -13201,7 +13207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="86" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B86" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B80),"",Prestations!B80)</f>
         <v/>
@@ -13232,7 +13238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="87" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B87" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B81),"",Prestations!B81)</f>
         <v/>
@@ -13263,7 +13269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="88" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B88" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B82),"",Prestations!B82)</f>
         <v/>
@@ -13294,7 +13300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="89" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B89" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B83),"",Prestations!B83)</f>
         <v/>
@@ -13325,7 +13331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="90" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B90" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B84),"",Prestations!B84)</f>
         <v/>
@@ -13356,7 +13362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="91" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B91" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B85),"",Prestations!B85)</f>
         <v/>
@@ -13387,7 +13393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="92" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B92" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B86),"",Prestations!B86)</f>
         <v/>
@@ -13418,7 +13424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="93" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B93" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B87),"",Prestations!B87)</f>
         <v/>
@@ -13452,7 +13458,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="94" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="94" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B94" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B88),"",Prestations!B88)</f>
         <v/>
@@ -13483,7 +13489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="95" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B95" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B89),"",Prestations!B89)</f>
         <v/>
@@ -13514,7 +13520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="96" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B96" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B90),"",Prestations!B90)</f>
         <v/>
@@ -13545,7 +13551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="97" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B97" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B91),"",Prestations!B91)</f>
         <v/>
@@ -13576,7 +13582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="98" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B98" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B92),"",Prestations!B92)</f>
         <v/>
@@ -13607,7 +13613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="99" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B99" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B93),"",Prestations!B93)</f>
         <v/>
@@ -13638,7 +13644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="100" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B100" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B94),"",Prestations!B94)</f>
         <v/>
@@ -13669,7 +13675,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="101" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B101" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B95),"",Prestations!B95)</f>
         <v/>
@@ -13703,7 +13709,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="102" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="102" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B102" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B96),"",Prestations!B96)</f>
         <v/>
@@ -13734,7 +13740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="103" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B103" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B97),"",Prestations!B97)</f>
         <v/>
@@ -13765,7 +13771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="104" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B104" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B98),"",Prestations!B98)</f>
         <v/>
@@ -13796,7 +13802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="105" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B105" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B99),"",Prestations!B99)</f>
         <v/>
@@ -13827,7 +13833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="106" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B106" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B100),"",Prestations!B100)</f>
         <v/>
@@ -13858,7 +13864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="107" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B107" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B101),"",Prestations!B101)</f>
         <v/>
@@ -13889,7 +13895,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="108" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B108" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B102),"",Prestations!B102)</f>
         <v/>
@@ -13920,7 +13926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="109" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B109" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B103),"",Prestations!B103)</f>
         <v/>
@@ -13951,7 +13957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="110" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B110" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B104),"",Prestations!B104)</f>
         <v/>
@@ -13982,7 +13988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="111" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B111" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B105),"",Prestations!B105)</f>
         <v/>
@@ -14013,7 +14019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="2:14" x14ac:dyDescent="0.35">
+    <row r="112" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B112" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B106),"",Prestations!B106)</f>
         <v/>
@@ -14044,7 +14050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B113" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B107),"",Prestations!B107)</f>
         <v/>
@@ -14075,7 +14081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B114" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B108),"",Prestations!B108)</f>
         <v/>
@@ -14106,7 +14112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B115" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B109),"",Prestations!B109)</f>
         <v/>
@@ -14137,7 +14143,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="116" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B116" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B110),"",Prestations!B110)</f>
         <v/>
@@ -14168,7 +14174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B117" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B111),"",Prestations!B111)</f>
         <v/>
@@ -14199,7 +14205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B118" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B112),"",Prestations!B112)</f>
         <v/>
@@ -14230,7 +14236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="119" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B119" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B113),"",Prestations!B113)</f>
         <v/>
@@ -14261,7 +14267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B120" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B114),"",Prestations!B114)</f>
         <v/>
@@ -14292,7 +14298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B121" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B115),"",Prestations!B115)</f>
         <v/>
@@ -14323,7 +14329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B122" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B116),"",Prestations!B116)</f>
         <v/>
@@ -14354,7 +14360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B123" s="107" t="str">
         <f>IF(ISBLANK(Prestations!B117),"",Prestations!B117)</f>
         <v/>
@@ -14385,7 +14391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="124" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B124" s="110" t="str">
         <f>IF(ISBLANK(Prestations!B118),"",Prestations!B118)</f>
         <v/>
@@ -14416,7 +14422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="125" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B125" s="91"/>
       <c r="C125" s="128" t="s">
         <v>28</v>
@@ -14431,7 +14437,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="2:12" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="126" spans="2:12" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B126" s="92"/>
       <c r="C126" s="165" t="str">
         <f>"Total à prendre en compte ("&amp;C6&amp;")"</f>
@@ -14447,14 +14453,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="2:12" x14ac:dyDescent="0.35"/>
-    <row r="128" spans="2:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="129" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="130" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="131" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="132" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="133" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="140" x14ac:dyDescent="0.35"/>
+    <row r="127" spans="2:12" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="2:12" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="129" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="130" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="131" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="132" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="133" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="140" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="116">
     <mergeCell ref="C86:D86"/>
@@ -14586,15 +14592,15 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0964DC6D-2EDA-461C-BEAD-DF4D797DB69C}">
-  <dimension ref="A1:C52"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C53"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="54.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="93.7265625" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="54.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="93.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>51</v>
       </c>
@@ -14602,7 +14608,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="98" t="s">
         <v>52</v>
       </c>
@@ -14613,7 +14619,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="119" t="s">
         <v>55</v>
       </c>
@@ -14621,7 +14627,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="119" t="s">
         <v>57</v>
       </c>
@@ -14629,7 +14635,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="119" t="s">
         <v>59</v>
       </c>
@@ -14637,7 +14643,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="119" t="s">
         <v>61</v>
       </c>
@@ -14645,7 +14651,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="119" t="s">
         <v>63</v>
       </c>
@@ -14653,7 +14659,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="119" t="s">
         <v>65</v>
       </c>
@@ -14661,7 +14667,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="119" t="s">
         <v>67</v>
       </c>
@@ -14669,7 +14675,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="119" t="s">
         <v>69</v>
       </c>
@@ -14677,7 +14683,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="119" t="s">
         <v>71</v>
       </c>
@@ -14685,7 +14691,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="119" t="s">
         <v>73</v>
       </c>
@@ -14693,7 +14699,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="119" t="s">
         <v>75</v>
       </c>
@@ -14701,7 +14707,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="119" t="s">
         <v>77</v>
       </c>
@@ -14709,7 +14715,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="119" t="s">
         <v>79</v>
       </c>
@@ -14717,7 +14723,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="119" t="s">
         <v>81</v>
       </c>
@@ -14725,7 +14731,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="119" t="s">
         <v>83</v>
       </c>
@@ -14733,7 +14739,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="119" t="s">
         <v>85</v>
       </c>
@@ -14741,7 +14747,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="119" t="s">
         <v>87</v>
       </c>
@@ -14749,7 +14755,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="119" t="s">
         <v>89</v>
       </c>
@@ -14757,7 +14763,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="119" t="s">
         <v>91</v>
       </c>
@@ -14765,7 +14771,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="119" t="s">
         <v>93</v>
       </c>
@@ -14773,7 +14779,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="119" t="s">
         <v>95</v>
       </c>
@@ -14781,7 +14787,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="119" t="s">
         <v>97</v>
       </c>
@@ -14789,7 +14795,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="119" t="s">
         <v>99</v>
       </c>
@@ -14797,7 +14803,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="119" t="s">
         <v>101</v>
       </c>
@@ -14805,7 +14811,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="119" t="s">
         <v>103</v>
       </c>
@@ -14813,7 +14819,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="119" t="s">
         <v>105</v>
       </c>
@@ -14821,7 +14827,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="119" t="s">
         <v>107</v>
       </c>
@@ -14829,7 +14835,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="119" t="s">
         <v>109</v>
       </c>
@@ -14837,7 +14843,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="119" t="s">
         <v>111</v>
       </c>
@@ -14845,7 +14851,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="119" t="s">
         <v>113</v>
       </c>
@@ -14853,7 +14859,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="119" t="s">
         <v>115</v>
       </c>
@@ -14861,7 +14867,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="119" t="s">
         <v>117</v>
       </c>
@@ -14869,7 +14875,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="119" t="s">
         <v>119</v>
       </c>
@@ -14877,7 +14883,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="119" t="s">
         <v>120</v>
       </c>
@@ -14885,7 +14891,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="119" t="s">
         <v>122</v>
       </c>
@@ -14893,7 +14899,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="119" t="s">
         <v>124</v>
       </c>
@@ -14901,7 +14907,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="119" t="s">
         <v>126</v>
       </c>
@@ -14909,7 +14915,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="119" t="s">
         <v>128</v>
       </c>
@@ -14917,7 +14923,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="119" t="s">
         <v>130</v>
       </c>
@@ -14925,7 +14931,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="119" t="s">
         <v>132</v>
       </c>
@@ -14933,7 +14939,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="119" t="s">
         <v>134</v>
       </c>
@@ -14941,7 +14947,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="119" t="s">
         <v>136</v>
       </c>
@@ -14949,7 +14955,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="119" t="s">
         <v>138</v>
       </c>
@@ -14957,7 +14963,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="119" t="s">
         <v>139</v>
       </c>
@@ -14965,7 +14971,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="119" t="s">
         <v>141</v>
       </c>
@@ -14973,7 +14979,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="119" t="s">
         <v>143</v>
       </c>
@@ -14981,7 +14987,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="119" t="s">
         <v>145</v>
       </c>
@@ -14989,7 +14995,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="119" t="s">
         <v>147</v>
       </c>
@@ -14997,7 +15003,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="119" t="s">
         <v>149</v>
       </c>
@@ -15005,12 +15011,20 @@
         <v>150</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="119" t="s">
         <v>151</v>
       </c>
       <c r="B52" s="119" t="s">
         <v>152</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="119" t="s">
+        <v>154</v>
+      </c>
+      <c r="B53" s="119" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -15023,12 +15037,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -15037,7 +15045,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B508D4C03FC42C45BBE2ADBDD824EFC0" ma:contentTypeVersion="6" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="cfba5fd0854cdbabcab6d21b092fe2fe">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8f591286-7764-4e50-b23d-301cdbd57747" xmlns:ns3="da57b96b-6ddc-49f5-b0eb-116682813bea" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a49260de3527cb3d25b090592fa664a3" ns2:_="" ns3:_="">
     <xsd:import namespace="8f591286-7764-4e50-b23d-301cdbd57747"/>
@@ -15214,16 +15222,13 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B677F5C1-D9F6-4847-A992-FC8EE88AA5D9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32730E2-0FA4-48D2-96BD-308CD4F34688}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -15231,7 +15236,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AACC739C-AFF3-49AC-B591-CFDB991CC673}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -15248,4 +15253,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B677F5C1-D9F6-4847-A992-FC8EE88AA5D9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>